<commit_message>
Fix error bar plus/minus element order so Excel shows them
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HfWi9EGRoRvmBivGaZdpwS
</commit_message>
<xml_diff>
--- a/three_sheets_line_charts.xlsx
+++ b/three_sheets_line_charts.xlsx
@@ -353,6 +353,27 @@
             <errBarType val="both"/>
             <errValType val="cust"/>
             <noEndCap val="0"/>
+            <plus>
+              <numRef>
+                <f>'正文所用数据 (2)'!$F$3:$F$6</f>
+                <numCache>
+                  <formatCode>General</formatCode>
+                  <ptCount val="4"/>
+                  <pt idx="0">
+                    <v>0</v>
+                  </pt>
+                  <pt idx="1">
+                    <v>1.732050807568877</v>
+                  </pt>
+                  <pt idx="2">
+                    <v>1.154700538379252</v>
+                  </pt>
+                  <pt idx="3">
+                    <v>2.309401076758503</v>
+                  </pt>
+                </numCache>
+              </numRef>
+            </plus>
             <minus>
               <numRef>
                 <f>'正文所用数据 (2)'!$F$3:$F$6</f>
@@ -374,27 +395,6 @@
                 </numCache>
               </numRef>
             </minus>
-            <plus>
-              <numRef>
-                <f>'正文所用数据 (2)'!$F$3:$F$6</f>
-                <numCache>
-                  <formatCode>General</formatCode>
-                  <ptCount val="4"/>
-                  <pt idx="0">
-                    <v>0</v>
-                  </pt>
-                  <pt idx="1">
-                    <v>1.732050807568877</v>
-                  </pt>
-                  <pt idx="2">
-                    <v>1.154700538379252</v>
-                  </pt>
-                  <pt idx="3">
-                    <v>2.309401076758503</v>
-                  </pt>
-                </numCache>
-              </numRef>
-            </plus>
             <spPr>
               <a:ln w="15000">
                 <a:solidFill>
@@ -481,6 +481,27 @@
             <errBarType val="both"/>
             <errValType val="cust"/>
             <noEndCap val="0"/>
+            <plus>
+              <numRef>
+                <f>'正文所用数据 (2)'!$F$9:$F$12</f>
+                <numCache>
+                  <formatCode>General</formatCode>
+                  <ptCount val="4"/>
+                  <pt idx="0">
+                    <v>1.732050807568877</v>
+                  </pt>
+                  <pt idx="1">
+                    <v>2.309401076758503</v>
+                  </pt>
+                  <pt idx="2">
+                    <v>2.309401076758503</v>
+                  </pt>
+                  <pt idx="3">
+                    <v>2.309401076758503</v>
+                  </pt>
+                </numCache>
+              </numRef>
+            </plus>
             <minus>
               <numRef>
                 <f>'正文所用数据 (2)'!$F$9:$F$12</f>
@@ -502,27 +523,6 @@
                 </numCache>
               </numRef>
             </minus>
-            <plus>
-              <numRef>
-                <f>'正文所用数据 (2)'!$F$9:$F$12</f>
-                <numCache>
-                  <formatCode>General</formatCode>
-                  <ptCount val="4"/>
-                  <pt idx="0">
-                    <v>1.732050807568877</v>
-                  </pt>
-                  <pt idx="1">
-                    <v>2.309401076758503</v>
-                  </pt>
-                  <pt idx="2">
-                    <v>2.309401076758503</v>
-                  </pt>
-                  <pt idx="3">
-                    <v>2.309401076758503</v>
-                  </pt>
-                </numCache>
-              </numRef>
-            </plus>
             <spPr>
               <a:ln w="15000">
                 <a:solidFill>
@@ -703,6 +703,27 @@
             <errBarType val="both"/>
             <errValType val="cust"/>
             <noEndCap val="0"/>
+            <plus>
+              <numRef>
+                <f>'正文所用数据'!$N$3:$N$6</f>
+                <numCache>
+                  <formatCode>General</formatCode>
+                  <ptCount val="4"/>
+                  <pt idx="0">
+                    <v>1.923538406167134</v>
+                  </pt>
+                  <pt idx="1">
+                    <v>2.792848008753789</v>
+                  </pt>
+                  <pt idx="2">
+                    <v>3.646916505762094</v>
+                  </pt>
+                  <pt idx="3">
+                    <v>3.03315017762062</v>
+                  </pt>
+                </numCache>
+              </numRef>
+            </plus>
             <minus>
               <numRef>
                 <f>'正文所用数据'!$N$3:$N$6</f>
@@ -724,27 +745,6 @@
                 </numCache>
               </numRef>
             </minus>
-            <plus>
-              <numRef>
-                <f>'正文所用数据'!$N$3:$N$6</f>
-                <numCache>
-                  <formatCode>General</formatCode>
-                  <ptCount val="4"/>
-                  <pt idx="0">
-                    <v>1.923538406167134</v>
-                  </pt>
-                  <pt idx="1">
-                    <v>2.792848008753789</v>
-                  </pt>
-                  <pt idx="2">
-                    <v>3.646916505762094</v>
-                  </pt>
-                  <pt idx="3">
-                    <v>3.03315017762062</v>
-                  </pt>
-                </numCache>
-              </numRef>
-            </plus>
             <spPr>
               <a:ln w="15000">
                 <a:solidFill>
@@ -831,6 +831,27 @@
             <errBarType val="both"/>
             <errValType val="cust"/>
             <noEndCap val="0"/>
+            <plus>
+              <numRef>
+                <f>'正文所用数据'!$N$9:$N$12</f>
+                <numCache>
+                  <formatCode>General</formatCode>
+                  <ptCount val="4"/>
+                  <pt idx="0">
+                    <v>2.190890230020665</v>
+                  </pt>
+                  <pt idx="1">
+                    <v>3.420526275297414</v>
+                  </pt>
+                  <pt idx="2">
+                    <v>2.683281572999748</v>
+                  </pt>
+                  <pt idx="3">
+                    <v>2.774887385102321</v>
+                  </pt>
+                </numCache>
+              </numRef>
+            </plus>
             <minus>
               <numRef>
                 <f>'正文所用数据'!$N$9:$N$12</f>
@@ -852,27 +873,6 @@
                 </numCache>
               </numRef>
             </minus>
-            <plus>
-              <numRef>
-                <f>'正文所用数据'!$N$9:$N$12</f>
-                <numCache>
-                  <formatCode>General</formatCode>
-                  <ptCount val="4"/>
-                  <pt idx="0">
-                    <v>2.190890230020665</v>
-                  </pt>
-                  <pt idx="1">
-                    <v>3.420526275297414</v>
-                  </pt>
-                  <pt idx="2">
-                    <v>2.683281572999748</v>
-                  </pt>
-                  <pt idx="3">
-                    <v>2.774887385102321</v>
-                  </pt>
-                </numCache>
-              </numRef>
-            </plus>
             <spPr>
               <a:ln w="15000">
                 <a:solidFill>
@@ -1053,6 +1053,33 @@
             <errBarType val="both"/>
             <errValType val="cust"/>
             <noEndCap val="0"/>
+            <plus>
+              <numRef>
+                <f>'正文所用数据 (3)'!$O$16:$O$21</f>
+                <numCache>
+                  <formatCode>General</formatCode>
+                  <ptCount val="6"/>
+                  <pt idx="0">
+                    <v>0.2081665999466132</v>
+                  </pt>
+                  <pt idx="1">
+                    <v>0.1527525231651946</v>
+                  </pt>
+                  <pt idx="2">
+                    <v>0.1732050807568876</v>
+                  </pt>
+                  <pt idx="3">
+                    <v>0.2645751311064591</v>
+                  </pt>
+                  <pt idx="4">
+                    <v>0.4041451884327379</v>
+                  </pt>
+                  <pt idx="5">
+                    <v>1</v>
+                  </pt>
+                </numCache>
+              </numRef>
+            </plus>
             <minus>
               <numRef>
                 <f>'正文所用数据 (3)'!$O$16:$O$21</f>
@@ -1080,33 +1107,6 @@
                 </numCache>
               </numRef>
             </minus>
-            <plus>
-              <numRef>
-                <f>'正文所用数据 (3)'!$O$16:$O$21</f>
-                <numCache>
-                  <formatCode>General</formatCode>
-                  <ptCount val="6"/>
-                  <pt idx="0">
-                    <v>0.2081665999466132</v>
-                  </pt>
-                  <pt idx="1">
-                    <v>0.1527525231651946</v>
-                  </pt>
-                  <pt idx="2">
-                    <v>0.1732050807568876</v>
-                  </pt>
-                  <pt idx="3">
-                    <v>0.2645751311064591</v>
-                  </pt>
-                  <pt idx="4">
-                    <v>0.4041451884327379</v>
-                  </pt>
-                  <pt idx="5">
-                    <v>1</v>
-                  </pt>
-                </numCache>
-              </numRef>
-            </plus>
             <spPr>
               <a:ln w="15000">
                 <a:solidFill>
@@ -1205,6 +1205,33 @@
             <errBarType val="both"/>
             <errValType val="cust"/>
             <noEndCap val="0"/>
+            <plus>
+              <numRef>
+                <f>'正文所用数据 (3)'!$Q$16:$Q$21</f>
+                <numCache>
+                  <formatCode>General</formatCode>
+                  <ptCount val="6"/>
+                  <pt idx="0">
+                    <v>0.5773502691896257</v>
+                  </pt>
+                  <pt idx="1">
+                    <v>0.5773502691896258</v>
+                  </pt>
+                  <pt idx="2">
+                    <v>0.5773502691896258</v>
+                  </pt>
+                  <pt idx="3">
+                    <v>0.5773502691896258</v>
+                  </pt>
+                  <pt idx="4">
+                    <v>0.5773502691896258</v>
+                  </pt>
+                  <pt idx="5">
+                    <v>1</v>
+                  </pt>
+                </numCache>
+              </numRef>
+            </plus>
             <minus>
               <numRef>
                 <f>'正文所用数据 (3)'!$Q$16:$Q$21</f>
@@ -1232,33 +1259,6 @@
                 </numCache>
               </numRef>
             </minus>
-            <plus>
-              <numRef>
-                <f>'正文所用数据 (3)'!$Q$16:$Q$21</f>
-                <numCache>
-                  <formatCode>General</formatCode>
-                  <ptCount val="6"/>
-                  <pt idx="0">
-                    <v>0.5773502691896257</v>
-                  </pt>
-                  <pt idx="1">
-                    <v>0.5773502691896258</v>
-                  </pt>
-                  <pt idx="2">
-                    <v>0.5773502691896258</v>
-                  </pt>
-                  <pt idx="3">
-                    <v>0.5773502691896258</v>
-                  </pt>
-                  <pt idx="4">
-                    <v>0.5773502691896258</v>
-                  </pt>
-                  <pt idx="5">
-                    <v>1</v>
-                  </pt>
-                </numCache>
-              </numRef>
-            </plus>
             <spPr>
               <a:ln w="15000">
                 <a:solidFill>
@@ -1357,6 +1357,33 @@
             <errBarType val="both"/>
             <errValType val="cust"/>
             <noEndCap val="0"/>
+            <plus>
+              <numRef>
+                <f>'正文所用数据 (3)'!$S$16:$S$21</f>
+                <numCache>
+                  <formatCode>General</formatCode>
+                  <ptCount val="6"/>
+                  <pt idx="0">
+                    <v>1</v>
+                  </pt>
+                  <pt idx="1">
+                    <v>1</v>
+                  </pt>
+                  <pt idx="2">
+                    <v>1</v>
+                  </pt>
+                  <pt idx="3">
+                    <v>1.527525231651947</v>
+                  </pt>
+                  <pt idx="4">
+                    <v>1</v>
+                  </pt>
+                  <pt idx="5">
+                    <v>1</v>
+                  </pt>
+                </numCache>
+              </numRef>
+            </plus>
             <minus>
               <numRef>
                 <f>'正文所用数据 (3)'!$S$16:$S$21</f>
@@ -1384,33 +1411,6 @@
                 </numCache>
               </numRef>
             </minus>
-            <plus>
-              <numRef>
-                <f>'正文所用数据 (3)'!$S$16:$S$21</f>
-                <numCache>
-                  <formatCode>General</formatCode>
-                  <ptCount val="6"/>
-                  <pt idx="0">
-                    <v>1</v>
-                  </pt>
-                  <pt idx="1">
-                    <v>1</v>
-                  </pt>
-                  <pt idx="2">
-                    <v>1</v>
-                  </pt>
-                  <pt idx="3">
-                    <v>1.527525231651947</v>
-                  </pt>
-                  <pt idx="4">
-                    <v>1</v>
-                  </pt>
-                  <pt idx="5">
-                    <v>1</v>
-                  </pt>
-                </numCache>
-              </numRef>
-            </plus>
             <spPr>
               <a:ln w="15000">
                 <a:solidFill>

</xml_diff>